<commit_message>
stage26: stabilize V37 runtime and A3 references
</commit_message>
<xml_diff>
--- a/lithosite-Mine-Services/Database/Mine-Services-Database-A3.xlsx
+++ b/lithosite-Mine-Services/Database/Mine-Services-Database-A3.xlsx
@@ -945,7 +945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1977,6 +1977,517 @@
       <c r="H26" t="inlineStr">
         <is>
           <t>v33-a3-delete-marker</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>779932f6-c7e0-4721-9bf2-70b9edaea566</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-10-05T01:42:21.191989+00:00</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>EQ-20261005-XR6Q</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>CREATE</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>{"category": "Heavy Equipment", "effective_from": "2026-10-01", "effective_to": null, "equipment_id": "EQ-20261005-XR6Q", "owner_name": "KPI Functional Test", "owner_type": "Owner", "status": "Active", "type": "Excavator", "unit_no": "EXCA-KPI-TEST-001"}</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>runtime-1791164541150-hun6pdh</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>01d638c2-baee-43fd-98c2-71d5e8946863</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-10-05T01:47:42.565551+00:00</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>OPS-20261005-TH9C5Q</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>CREATE</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>{"activity": "Digging", "actual_hours": 4, "created_at": "2026-10-05T01:47:42.564813+00:00", "domain": "Road &amp; Hauling", "equipment_id": "EQ-20261005-XR6Q", "quantity": 100, "source": "Manual", "status": "VALIDATED", "target_hours": 4, "transaction_date": "2026-10-01", "transaction_id": "OPS-20261005-TH9C5Q", "transaction_time": "06:00", "unit": "ton", "updated_at": "2026-10-05T01:47:42.564813+00:00", "work_front_id": "WF-20260930-EGB1"}</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>runtime-1791164862557-593vfu2</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>46a90d3e-f5f0-4c0c-b059-cbaf53dec029</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-10-05T01:53:06.459997+00:00</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>OPS-20261005-HNQJBI</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>CREATE</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>{"activity": "Normal spotting", "actual_hours": 1, "created_at": "2026-10-05T01:53:06.459354+00:00", "domain": "Road &amp; Hauling", "equipment_id": "EQ-20261005-XR6Q", "quantity": 10, "source": "Manual", "status": "VALIDATED", "target_hours": 1, "transaction_date": "2026-10-01", "transaction_id": "OPS-20261005-HNQJBI", "transaction_time": "10:00", "unit": "ton", "updated_at": "2026-10-05T01:53:06.459354+00:00", "work_front_id": "WF-20260930-EGB1"}</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>runtime-1791165186455-nsrj9vl</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>50229784-0045-43e9-850c-0395d29c8f53</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:04:41.165800+00:00</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>OPS-20261005-3N43EV</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>CREATE</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>{"activity": "Loading1", "actual_hours": 1, "created_at": "2026-10-05T02:04:41.164835+00:00", "domain": "Road &amp; Hauling", "equipment_id": "EQ-20261005-XR6Q", "quantity": 100, "source": "Manual", "status": "VALIDATED", "target_hours": 1, "transaction_date": "2026-10-01", "transaction_id": "OPS-20261005-3N43EV", "transaction_time": "10:00", "unit": "ton", "updated_at": "2026-10-05T02:04:41.164835+00:00", "work_front_id": "WF-20260930-EGB1"}</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>runtime-1791165881160-tx595cm</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>7110d39f-c2fd-4b48-ba36-4820261a9e67</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:04:50.369190+00:00</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>OPS-20261005-3N43EV</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>UPDATE</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>{"activity": "Loading1", "actual_hours": 1, "created_at": "2026-10-05T02:04:41.164835+00:00", "domain": "Road &amp; Hauling", "equipment_id": "EQ-20261005-XR6Q", "quantity": 100, "source": "Manual", "status": "VALIDATED", "target_hours": 1, "transaction_date": "2026-10-01", "transaction_id": "OPS-20261005-3N43EV", "transaction_time": "10:00", "unit": "ton", "updated_at": "2026-10-05T02:04:41.164835+00:00", "work_front_id": "WF-20260930-EGB1"}</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>{"activity": "Loading", "actual_hours": 1, "created_at": "2026-10-05T02:04:41.164835+00:00", "domain": "Road &amp; Hauling", "equipment_id": "EQ-20261005-XR6Q", "quantity": 100, "source": "Manual", "status": "VALIDATED", "target_hours": 1, "transaction_date": "2026-10-01", "transaction_id": "OPS-20261005-3N43EV", "transaction_time": "10:00", "unit": "ton", "updated_at": "2026-10-05T02:04:50.368306+00:00", "work_front_id": "WF-20260930-EGB1"}</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>runtime-1791165890362-0nc6ic2</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>314ddae3-6a12-48bb-b2d8-6408ece265f1</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:05:52.120290+00:00</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>OPS-20261005-3N43EV</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>UPDATE</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>{"activity": "Loading", "actual_hours": 1, "created_at": "2026-10-05T02:04:41.164835+00:00", "domain": "Road &amp; Hauling", "equipment_id": "EQ-20261005-XR6Q", "quantity": 100, "source": "Manual", "status": "VALIDATED", "target_hours": 1, "transaction_date": "2026-10-01", "transaction_id": "OPS-20261005-3N43EV", "transaction_time": "10:00", "unit": "ton", "updated_at": "2026-10-05T02:04:50.368306+00:00", "work_front_id": "WF-20260930-EGB1"}</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>{"activity": "Loading", "actual_hours": 1, "created_at": "2026-10-05T02:04:41.164835+00:00", "domain": "Road &amp; Hauling", "equipment_id": "EQ-20261005-XR6Q", "quantity": 100, "source": "Manual", "status": "VALIDATED", "target_hours": 1, "transaction_date": "2026-10-01", "transaction_id": "OPS-20261005-3N43EV", "transaction_time": "11:00", "unit": "ton", "updated_at": "2026-10-05T02:05:52.119099+00:00", "work_front_id": "WF-20260930-EGB1"}</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>runtime-1791165952114-j8jm5ib</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>06c22cce-9148-47dc-8d02-cb1729f25f2e</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:09:08.451014+00:00</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>OPS-20261005-47Y7K6</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>CREATE</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>{"activity": "Digging", "actual_hours": 3, "created_at": "2026-10-05T02:09:08.450102+00:00", "domain": "Road &amp; Hauling", "equipment_id": "EQ-20261005-XR6Q", "quantity": 100, "source": "Manual", "status": "VALIDATED", "target_hours": 3, "transaction_date": "2026-10-01", "transaction_id": "OPS-20261005-47Y7K6", "transaction_time": "09:08", "unit": "ton", "updated_at": "2026-10-05T02:09:08.450102+00:00", "work_front_id": "WF-20260930-EGB1"}</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>runtime-1791166148443-qctdbpd</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>fa7488f4-f261-48b0-a907-2cffbe10011e</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:09:27.064851+00:00</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>OPS-20261005-47Y7K6</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>UPDATE</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>{"activity": "Digging", "actual_hours": 3, "created_at": "2026-10-05T02:09:08.450102+00:00", "domain": "Road &amp; Hauling", "equipment_id": "EQ-20261005-XR6Q", "quantity": 100, "source": "Manual", "status": "VALIDATED", "target_hours": 3, "transaction_date": "2026-10-01", "transaction_id": "OPS-20261005-47Y7K6", "transaction_time": "09:08", "unit": "ton", "updated_at": "2026-10-05T02:09:08.450102+00:00", "work_front_id": "WF-20260930-EGB1"}</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>{"activity": "Digging", "actual_hours": 3, "created_at": "2026-10-05T02:09:08.450102+00:00", "domain": "Road &amp; Hauling", "equipment_id": "EQ-20261005-XR6Q", "quantity": 100, "source": "Manual", "status": "VALIDATED", "target_hours": 3, "transaction_date": "2026-10-01", "transaction_id": "OPS-20261005-47Y7K6", "transaction_time": "01:00", "unit": "ton", "updated_at": "2026-10-05T02:09:27.064083+00:00", "work_front_id": "WF-20260930-EGB1"}</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>runtime-1791166167057-3bw7pl5</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>0e630aa5-9610-4b46-914f-2dfba42b6334</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:13:33.558252+00:00</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>OPS-20261005-47Y7K6</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>UPDATE</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>{"activity": "Digging", "actual_hours": 3, "created_at": "2026-10-05T02:09:08.450102+00:00", "domain": "Road &amp; Hauling", "equipment_id": "EQ-20261005-XR6Q", "quantity": 100, "source": "Manual", "status": "VALIDATED", "target_hours": 3, "transaction_date": "2026-10-01", "transaction_id": "OPS-20261005-47Y7K6", "transaction_time": "01:00", "unit": "ton", "updated_at": "2026-10-05T02:09:27.064083+00:00", "work_front_id": "WF-20260930-EGB1"}</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>{"activity": "Digging", "actual_hours": 3, "created_at": "2026-10-05T02:09:08.450102+00:00", "domain": "Road &amp; Hauling", "equipment_id": "EQ-20261005-XR6Q", "quantity": 100, "source": "Manual", "status": "VALIDATED", "target_hours": 3, "transaction_date": "2026-10-01", "transaction_id": "OPS-20261005-47Y7K6", "transaction_time": "13:00", "unit": "ton", "updated_at": "2026-10-05T02:13:33.557253+00:00", "work_front_id": "WF-20260930-EGB1"}</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>runtime-1791166413550-vrb7qoh</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>871affeb-e0c2-479f-9ad4-1c25ca89d7c3</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:15:32.870618+00:00</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>OPS-20261005-X29LW8</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>CREATE</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>{"activity": "Loading", "actual_hours": 2, "created_at": "2026-10-05T02:15:32.870039+00:00", "domain": "Road &amp; Hauling", "equipment_id": "EQ-20261005-XR6Q", "quantity": 100, "source": "Manual", "status": "VALIDATED", "target_hours": 2, "transaction_date": "2026-10-01", "transaction_id": "OPS-20261005-X29LW8", "transaction_time": "16:14", "unit": "ton", "updated_at": "2026-10-05T02:15:32.870039+00:00", "work_front_id": "WF-20260930-EGB1"}</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>runtime-1791166532863-xt306hb</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>82c96d1c-da31-4726-b5ff-b9bab5822c2c</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:17:03.798029+00:00</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>OPS-20261005-X29LW8</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>UPDATE</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>{"activity": "Loading", "actual_hours": 2, "created_at": "2026-10-05T02:15:32.870039+00:00", "domain": "Road &amp; Hauling", "equipment_id": "EQ-20261005-XR6Q", "quantity": 100, "source": "Manual", "status": "VALIDATED", "target_hours": 2, "transaction_date": "2026-10-01", "transaction_id": "OPS-20261005-X29LW8", "transaction_time": "16:14", "unit": "ton", "updated_at": "2026-10-05T02:15:32.870039+00:00", "work_front_id": "WF-20260930-EGB1"}</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>{"activity": "Loading", "actual_hours": 2, "created_at": "2026-10-05T02:15:32.870039+00:00", "domain": "Road &amp; Hauling", "equipment_id": "EQ-20261005-XR6Q", "quantity": 100, "source": "Manual", "status": "VALIDATED", "target_hours": 2, "transaction_date": "2026-10-01", "transaction_id": "OPS-20261005-X29LW8", "transaction_time": "16:00", "unit": "ton", "updated_at": "2026-10-05T02:17:03.797036+00:00", "work_front_id": "WF-20260930-EGB1"}</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>runtime-1791166623790-irpvr6k</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>38c9812f-84a2-440b-b8d9-6ad8138a15c9</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:36:03.780828+00:00</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>EQ-20261005-T7XQ</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>CREATE</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>{"category": "Heavy Equipment", "effective_from": "2026-10-02", "effective_to": null, "equipment_id": "EQ-20261005-T7XQ", "owner_name": "Ruli", "owner_type": "Owner", "status": "Active", "type": "Dozer", "unit_no": "DZR-KPI-TEST-001"}</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>runtime-1791167763776-mju1mf4</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>3d03185f-fefb-4237-8fbd-f76afcfddd03</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:36:21.722748+00:00</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>EQ-20261005-T7XQ</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>UPDATE</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>{"category": "Heavy Equipment", "effective_from": "2026-10-02", "effective_to": null, "equipment_id": "EQ-20261005-T7XQ", "owner_name": "Ruli", "owner_type": "Owner", "status": "Active", "type": "Dozer", "unit_no": "DZR-KPI-TEST-001"}</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>{"category": "Heavy Equipment", "effective_from": "2026-10-02", "effective_to": null, "equipment_id": "EQ-20261005-T7XQ", "owner_name": "KPI Functional Test", "owner_type": "Owner", "status": "Active", "type": "Dozer", "unit_no": "DZR-KPI-TEST-001"}</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>runtime-1791167781716-i7lmb81</t>
         </is>
       </c>
     </row>
@@ -2705,6 +3216,11 @@
           <t>Light Vehicle</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Mining</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>unit</t>
@@ -2720,6 +3236,11 @@
       <c r="B9" t="inlineStr">
         <is>
           <t>Other</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>cycle</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -2739,7 +3260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2922,6 +3443,90 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>2026-10-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>EQ-20261005-XR6Q</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>EXCA-KPI-TEST-001</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Heavy Equipment</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Excavator</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>KPI Functional Test</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>EQ-20261005-T7XQ</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DZR-KPI-TEST-001</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Heavy Equipment</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Dozer</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>KPI Functional Test</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -3056,7 +3661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3292,6 +3897,361 @@
       <c r="O3" t="inlineStr">
         <is>
           <t>2026-09-30T22:48:57.047012+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>OPS-20261005-TH9C5Q</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Road &amp; Hauling</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>WF-20260930-EGB1</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>EQ-20261005-XR6Q</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Digging</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>100</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ton</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>VALIDATED</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2026-10-05T01:47:42.564813+00:00</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>2026-10-05T01:47:42.564813+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>OPS-20261005-HNQJBI</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Road &amp; Hauling</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>WF-20260930-EGB1</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>EQ-20261005-XR6Q</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Normal spotting</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>10</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>ton</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>VALIDATED</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2026-10-05T01:53:06.459354+00:00</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>2026-10-05T01:53:06.459354+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>OPS-20261005-3N43EV</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Road &amp; Hauling</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>WF-20260930-EGB1</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>EQ-20261005-XR6Q</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>100</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>ton</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>VALIDATED</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:04:41.164835+00:00</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:05:52.119099+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>OPS-20261005-47Y7K6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Road &amp; Hauling</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>WF-20260930-EGB1</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>EQ-20261005-XR6Q</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Digging</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>100</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>ton</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>3</v>
+      </c>
+      <c r="K7" t="n">
+        <v>3</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>VALIDATED</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:09:08.450102+00:00</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:13:33.557253+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>OPS-20261005-X29LW8</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Road &amp; Hauling</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>WF-20260930-EGB1</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>EQ-20261005-XR6Q</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Loading</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>100</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>ton</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>VALIDATED</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:15:32.870039+00:00</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>2026-10-05T02:17:03.797036+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>